<commit_message>
Add super-admin dry-run testing, alef name matching, and student roster update.
Allow Telegram ID 94571452 to complete verification and receive credentials without writing claim data; treat آ and ا as equivalent in name matching; shorten the contact prompt; ship the updated Stdnts-all.xlsx.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Stdnts-all.xlsx
+++ b/Stdnts-all.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhzd/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhzd/Desktop/UT - Courses/Students-Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{145823DC-6C99-BA49-B68E-5D8D6569D28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0895A82-73D2-2F43-AB59-2FF742730573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2780" yWindow="1500" windowWidth="28040" windowHeight="17440" xr2:uid="{84B7E3B6-4B67-244A-9395-A5C53FC92356}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{84B7E3B6-4B67-244A-9395-A5C53FC92356}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="405">
   <si>
     <t>4305042_02</t>
   </si>
@@ -621,6 +621,636 @@
   </si>
   <si>
     <t>https://exam.behzadminaei.ir/e/or-ex2/login</t>
+  </si>
+  <si>
+    <t>4303390_04</t>
+  </si>
+  <si>
+    <t>ادمي داريان درسا</t>
+  </si>
+  <si>
+    <t>A7mK2pQ9</t>
+  </si>
+  <si>
+    <t>اسماعيلي فاطمه</t>
+  </si>
+  <si>
+    <t>x4Bv8Nq1</t>
+  </si>
+  <si>
+    <t>اميري مينا</t>
+  </si>
+  <si>
+    <t>مديريت بيمه</t>
+  </si>
+  <si>
+    <t>R6tY3wL8</t>
+  </si>
+  <si>
+    <t>بازياري علي</t>
+  </si>
+  <si>
+    <t>c9Hj2Msa</t>
+  </si>
+  <si>
+    <t>حاجي ابراهيمي اول نرگس</t>
+  </si>
+  <si>
+    <t>P5dF7kZ3</t>
+  </si>
+  <si>
+    <t>حسيني ياسمين سادات</t>
+  </si>
+  <si>
+    <t>n8Qx4Vb6</t>
+  </si>
+  <si>
+    <t>ذهبيون ستايش</t>
+  </si>
+  <si>
+    <t>T2mR9cW5</t>
+  </si>
+  <si>
+    <t>زارعي فاطمه</t>
+  </si>
+  <si>
+    <t>g7Lk3Pz8</t>
+  </si>
+  <si>
+    <t>سليمانيون فاطمه</t>
+  </si>
+  <si>
+    <t>Y4sN6hJ2</t>
+  </si>
+  <si>
+    <t>سيدان ملك سيدعلي</t>
+  </si>
+  <si>
+    <t>b9Dq5Xr7</t>
+  </si>
+  <si>
+    <t>شكوري فائزه</t>
+  </si>
+  <si>
+    <t>K3vM8tA4</t>
+  </si>
+  <si>
+    <t>صدري ارغوان</t>
+  </si>
+  <si>
+    <t>w6Zp2Fj9</t>
+  </si>
+  <si>
+    <t>طاهري قمي سيدابوالفضل</t>
+  </si>
+  <si>
+    <t>H8cR4nY7</t>
+  </si>
+  <si>
+    <t>علي اقاپور اميرعباس</t>
+  </si>
+  <si>
+    <t>q2Gm9Lx5</t>
+  </si>
+  <si>
+    <t>غفوري ستايش</t>
+  </si>
+  <si>
+    <t>V7bT3kP8</t>
+  </si>
+  <si>
+    <t>كريمي نژاد ريحانه</t>
+  </si>
+  <si>
+    <t>d5Jw6Nz2</t>
+  </si>
+  <si>
+    <t>محرابي عليرضا</t>
+  </si>
+  <si>
+    <t>M9rC4sH7</t>
+  </si>
+  <si>
+    <t>محمدي سجاد</t>
+  </si>
+  <si>
+    <t>z3Xf8Qv1</t>
+  </si>
+  <si>
+    <t>مشهدي عبدالرحمن محمد</t>
+  </si>
+  <si>
+    <t>E6nK2yB9</t>
+  </si>
+  <si>
+    <t>مهربان جهرمي مائده</t>
+  </si>
+  <si>
+    <t>p4Wj7Td5</t>
+  </si>
+  <si>
+    <t>ناظمي سجزي عرفان</t>
+  </si>
+  <si>
+    <t>S8aL3mR6</t>
+  </si>
+  <si>
+    <t>نژديار حنانه</t>
+  </si>
+  <si>
+    <t>h2Vq9Fz4</t>
+  </si>
+  <si>
+    <t>يعقوبي مهسا</t>
+  </si>
+  <si>
+    <t>N7kD5xC8</t>
+  </si>
+  <si>
+    <t>https://exam.behzadminaei.ir/e/or2-ex/login</t>
+  </si>
+  <si>
+    <t>4301247_01</t>
+  </si>
+  <si>
+    <t>ادبي فيروزجائي كوثر</t>
+  </si>
+  <si>
+    <t>حسابداري</t>
+  </si>
+  <si>
+    <t>B7mQ2xK9</t>
+  </si>
+  <si>
+    <t>ادعاجو محمدرضا</t>
+  </si>
+  <si>
+    <t>v4N8pR1a</t>
+  </si>
+  <si>
+    <t>استوار ريحانه</t>
+  </si>
+  <si>
+    <t>T6yH3wL8</t>
+  </si>
+  <si>
+    <t>اسدالهي سيدايليا</t>
+  </si>
+  <si>
+    <t>c9Jk2MZ5</t>
+  </si>
+  <si>
+    <t>افشاري حسين</t>
+  </si>
+  <si>
+    <t>P5dF7nX3</t>
+  </si>
+  <si>
+    <t>اقبالي پريا</t>
+  </si>
+  <si>
+    <t>q8Vx4Bb6</t>
+  </si>
+  <si>
+    <t>اكبري سارا</t>
+  </si>
+  <si>
+    <t>R2mY9cW5</t>
+  </si>
+  <si>
+    <t>اكبري محمدحسين</t>
+  </si>
+  <si>
+    <t>g7Lh3Sz8</t>
+  </si>
+  <si>
+    <t>اميدي محدثه</t>
+  </si>
+  <si>
+    <t>K4sN6jT2</t>
+  </si>
+  <si>
+    <t>ايماني ندا</t>
+  </si>
+  <si>
+    <t>مديريت امور بانكي</t>
+  </si>
+  <si>
+    <t>b9Dq5Ar7</t>
+  </si>
+  <si>
+    <t>باقري گوراند محمدصدرا</t>
+  </si>
+  <si>
+    <t>M3vP8tH4</t>
+  </si>
+  <si>
+    <t>برخوردار فاطمه</t>
+  </si>
+  <si>
+    <t>w6Zk2Fj9</t>
+  </si>
+  <si>
+    <t>پيري اغوزبني ياسمن</t>
+  </si>
+  <si>
+    <t>جامعي محمد</t>
+  </si>
+  <si>
+    <t>x2Gm9Lq5</t>
+  </si>
+  <si>
+    <t>جودكي محمدمعين</t>
+  </si>
+  <si>
+    <t>V7bT3pK8</t>
+  </si>
+  <si>
+    <t>چوپاني مائده</t>
+  </si>
+  <si>
+    <t>حقيقت شعاراصل دريا</t>
+  </si>
+  <si>
+    <t>C9rM4sH7</t>
+  </si>
+  <si>
+    <t>خادمان امام رضا محيا</t>
+  </si>
+  <si>
+    <t>خداوردي محمدرضا</t>
+  </si>
+  <si>
+    <t>خلخالي نژادبندري پريسا</t>
+  </si>
+  <si>
+    <t>خليل ابادي صالح</t>
+  </si>
+  <si>
+    <t>خليلي حديث</t>
+  </si>
+  <si>
+    <t>دل شكيب حسنا</t>
+  </si>
+  <si>
+    <t>رسائي محي الدين</t>
+  </si>
+  <si>
+    <t>A3pY8mJ6</t>
+  </si>
+  <si>
+    <t>رضائي ياسر</t>
+  </si>
+  <si>
+    <t>r9Bv2Kq7</t>
+  </si>
+  <si>
+    <t>روزبهاني دلارام</t>
+  </si>
+  <si>
+    <t>F5xT4nZ8</t>
+  </si>
+  <si>
+    <t>روستائي اطهر</t>
+  </si>
+  <si>
+    <t>j7M3wP9c</t>
+  </si>
+  <si>
+    <t>روستائي محدثه</t>
+  </si>
+  <si>
+    <t>Q2dH6sL5</t>
+  </si>
+  <si>
+    <t>زارعي محمدرضا</t>
+  </si>
+  <si>
+    <t>u8Rk4Xb3</t>
+  </si>
+  <si>
+    <t>سرگردان فرداراني نيكا</t>
+  </si>
+  <si>
+    <t>G9mV7qA2</t>
+  </si>
+  <si>
+    <t>سيف الهي ستاره</t>
+  </si>
+  <si>
+    <t>t4Cz8Nf6</t>
+  </si>
+  <si>
+    <t>سيمياري مهديه</t>
+  </si>
+  <si>
+    <t>W6pJ3yK9</t>
+  </si>
+  <si>
+    <t>شكري فاطمه</t>
+  </si>
+  <si>
+    <t>n2Dq7Hvx</t>
+  </si>
+  <si>
+    <t>صباحي فرد مطهره</t>
+  </si>
+  <si>
+    <t>L8sF5mR4</t>
+  </si>
+  <si>
+    <t>صدري كوپائي تكتم</t>
+  </si>
+  <si>
+    <t>e3Tj9Bz7</t>
+  </si>
+  <si>
+    <t>صفرزاده محمد</t>
+  </si>
+  <si>
+    <t>X7kP2cN6</t>
+  </si>
+  <si>
+    <t>طحاني پور محمدمتين</t>
+  </si>
+  <si>
+    <t>a5Vw8Qm3</t>
+  </si>
+  <si>
+    <t>عبادي هانيه سادات</t>
+  </si>
+  <si>
+    <t>J9hR4xD7</t>
+  </si>
+  <si>
+    <t>عبدالحسيني قريه علي بهاره</t>
+  </si>
+  <si>
+    <t>f2Zk6Tn8</t>
+  </si>
+  <si>
+    <t>علي پورخالصي شيرازي مسيح</t>
+  </si>
+  <si>
+    <t>Y8qC3pL5</t>
+  </si>
+  <si>
+    <t>عليزاده شيما</t>
+  </si>
+  <si>
+    <t>m4Gv9Bs2</t>
+  </si>
+  <si>
+    <t>فريدوني اميررضا</t>
+  </si>
+  <si>
+    <t>K6xN7dW3</t>
+  </si>
+  <si>
+    <t>فصاحت رعنا</t>
+  </si>
+  <si>
+    <t>r3Hj8Qp5</t>
+  </si>
+  <si>
+    <t>فيضي ريحانه</t>
+  </si>
+  <si>
+    <t>P9tM2zF6</t>
+  </si>
+  <si>
+    <t>قاسمي فائزه</t>
+  </si>
+  <si>
+    <t>c7Lw4Vn8</t>
+  </si>
+  <si>
+    <t>قلي زاده سبحان</t>
+  </si>
+  <si>
+    <t>D5qY9kA3</t>
+  </si>
+  <si>
+    <t>ما لايك</t>
+  </si>
+  <si>
+    <t>s8Xb2Jm7</t>
+  </si>
+  <si>
+    <t>محبوب ايراني اميرمحمد</t>
+  </si>
+  <si>
+    <t>U4nR6pZ9</t>
+  </si>
+  <si>
+    <t>محمدي اسد حسنا</t>
+  </si>
+  <si>
+    <t>g9Fv3Kx5</t>
+  </si>
+  <si>
+    <t>مختاري عليرضا</t>
+  </si>
+  <si>
+    <t>B2mT8qH4</t>
+  </si>
+  <si>
+    <t>مظاهري محمدصادق</t>
+  </si>
+  <si>
+    <t>y7Cj5Wn3</t>
+  </si>
+  <si>
+    <t>مقيسه عليرضا</t>
+  </si>
+  <si>
+    <t>N4pL9dR6</t>
+  </si>
+  <si>
+    <t>موسوي كياناسادات</t>
+  </si>
+  <si>
+    <t>h6Qx3Vb8</t>
+  </si>
+  <si>
+    <t>مهراب پور رعنا</t>
+  </si>
+  <si>
+    <t>Z8kG2mT7</t>
+  </si>
+  <si>
+    <t>نظري سيده مبينا</t>
+  </si>
+  <si>
+    <t>w3Jf7Pq9</t>
+  </si>
+  <si>
+    <t>نظري شيوا</t>
+  </si>
+  <si>
+    <t>M5rD8yK2</t>
+  </si>
+  <si>
+    <t>نگه دارنيكو كمند</t>
+  </si>
+  <si>
+    <t>a9Vn4Xc6</t>
+  </si>
+  <si>
+    <t>نوروزي خاص غزل</t>
+  </si>
+  <si>
+    <t>T3bH7sL5</t>
+  </si>
+  <si>
+    <t>وهابي اذرخواراني مهدي</t>
+  </si>
+  <si>
+    <t>q6Zp2Fj8</t>
+  </si>
+  <si>
+    <t>https://exam.behzadminaei.ir/e/or-ex3/login</t>
+  </si>
+  <si>
+    <t>4308036_08</t>
+  </si>
+  <si>
+    <t>اسايش زارچي سيدمصطفي</t>
+  </si>
+  <si>
+    <t>R7mK2pX9</t>
+  </si>
+  <si>
+    <t>باقري اميرمحمد</t>
+  </si>
+  <si>
+    <t>b4Nq8Vt1</t>
+  </si>
+  <si>
+    <t>برزوئي دينا</t>
+  </si>
+  <si>
+    <t>H6yT3wL8</t>
+  </si>
+  <si>
+    <t>تاجيك رومينا</t>
+  </si>
+  <si>
+    <t>c9Jf2MZ5</t>
+  </si>
+  <si>
+    <t>تراب زاده ايليا</t>
+  </si>
+  <si>
+    <t>P5dG7nQ3</t>
+  </si>
+  <si>
+    <t>ترك چين محمدطاها</t>
+  </si>
+  <si>
+    <t>x8Vk4Bb6</t>
+  </si>
+  <si>
+    <t>تهمتن يگانه</t>
+  </si>
+  <si>
+    <t>T2mY9cR5</t>
+  </si>
+  <si>
+    <t>چشم الوس حسين</t>
+  </si>
+  <si>
+    <t>حبيبي محمد پارسا</t>
+  </si>
+  <si>
+    <t>K4sN6jW2</t>
+  </si>
+  <si>
+    <t>رافتي سخنگو سجاد</t>
+  </si>
+  <si>
+    <t>a9Dq5Fr7</t>
+  </si>
+  <si>
+    <t>سليمان او محمد جواد</t>
+  </si>
+  <si>
+    <t>سهرابي محمدعارف</t>
+  </si>
+  <si>
+    <t>w6Zk2Gj9</t>
+  </si>
+  <si>
+    <t>عارف لاله فاطمه</t>
+  </si>
+  <si>
+    <t>J8cR4nY7</t>
+  </si>
+  <si>
+    <t>عبادي طزرجاني يكتا</t>
+  </si>
+  <si>
+    <t>غلام پور محمدحسين</t>
+  </si>
+  <si>
+    <t>V7bT3pN8</t>
+  </si>
+  <si>
+    <t>قاسمي كنسي نسترن</t>
+  </si>
+  <si>
+    <t>d5Kw6Az2</t>
+  </si>
+  <si>
+    <t>قرباني اميرحسين</t>
+  </si>
+  <si>
+    <t>C9rM4sF7</t>
+  </si>
+  <si>
+    <t>قربانيان فاطمه</t>
+  </si>
+  <si>
+    <t>z3Xh8Qv1</t>
+  </si>
+  <si>
+    <t>كلايه نازنين زهرا</t>
+  </si>
+  <si>
+    <t>كولائي ساراي</t>
+  </si>
+  <si>
+    <t>محبعلي محدثه</t>
+  </si>
+  <si>
+    <t>محمدابادي علي</t>
+  </si>
+  <si>
+    <t>مختاري اميرعلي</t>
+  </si>
+  <si>
+    <t>مختوم عمر</t>
+  </si>
+  <si>
+    <t>مسعوديان سيداميرحسين</t>
+  </si>
+  <si>
+    <t>مفيدي نژاد امير</t>
+  </si>
+  <si>
+    <t>ولي الينا</t>
+  </si>
+  <si>
+    <t>هاشمي پرنيان</t>
+  </si>
+  <si>
+    <t>هاشمي حنانه</t>
+  </si>
+  <si>
+    <t>يعقوبيان ناره</t>
+  </si>
+  <si>
+    <t>https://exam.behzadminaei.ir/e/stats1-exam/login</t>
   </si>
 </sst>
 </file>
@@ -1023,14 +1653,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6278815-03C6-D044-88F9-6540261AD0A4}">
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.5" customWidth="1"/>
-    <col min="6" max="6" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -2851,6 +3481,2246 @@
       </c>
       <c r="F91" s="3" t="s">
         <v>194</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D92" s="1">
+        <v>433803055</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93" s="1">
+        <v>433803057</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D94" s="1">
+        <v>432201064</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95" s="1">
+        <v>433803061</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D96" s="1">
+        <v>433803068</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D97" s="1">
+        <v>432201033</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D98" s="1">
+        <v>432201035</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F98" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D99" s="1">
+        <v>433803072</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D100" s="1">
+        <v>430302099</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101" s="1">
+        <v>430301085</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F101" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D102" s="1">
+        <v>432201034</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D103" s="1">
+        <v>433803074</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D104" s="1">
+        <v>432201031</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D105" s="1">
+        <v>432201032</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D106" s="1">
+        <v>430302108</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D107" s="1">
+        <v>430302115</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D108" s="1">
+        <v>430501101</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D109" s="1">
+        <v>430301097</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D110" s="1">
+        <v>433803080</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D111" s="1">
+        <v>430302129</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D112" s="1">
+        <v>432201066</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D113" s="1">
+        <v>430302130</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D114" s="1">
+        <v>430302136</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D115" s="1">
+        <v>430103027</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D116" s="1">
+        <v>430103028</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D117" s="1">
+        <v>432202006</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D118" s="1">
+        <v>430103029</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D119" s="1">
+        <v>430103030</v>
+      </c>
+      <c r="E119" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D120" s="1">
+        <v>432202010</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D121" s="1">
+        <v>432202011</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D122" s="1">
+        <v>430103031</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D123" s="1">
+        <v>430102034</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D124" s="1">
+        <v>432203024</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D125" s="1">
+        <v>432203025</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A126" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D126" s="1">
+        <v>430103032</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A127" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D127" s="1">
+        <v>430103034</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D128" s="1">
+        <v>430103035</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D129" s="1">
+        <v>430103036</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D130" s="1">
+        <v>430103037</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D131" s="1">
+        <v>430103038</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D132" s="1">
+        <v>432202012</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D133" s="1">
+        <v>430103040</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A134" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D134" s="1">
+        <v>430103041</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A135" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D135" s="1">
+        <v>430103042</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F135" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D136" s="1">
+        <v>432202067</v>
+      </c>
+      <c r="E136" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="F136" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D137" s="1">
+        <v>433803091</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F137" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A138" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D138" s="1">
+        <v>430103043</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A139" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D139" s="1">
+        <v>430102042</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A140" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B140" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D140" s="1">
+        <v>430103044</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F140" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A141" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B141" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D141" s="1">
+        <v>430103045</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F141" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A142" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D142" s="1">
+        <v>430102044</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="F142" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A143" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B143" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D143" s="1">
+        <v>430103046</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A144" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B144" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D144" s="1">
+        <v>430103048</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="F144" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A145" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D145" s="1">
+        <v>430103049</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="F145" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A146" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D146" s="1">
+        <v>430103050</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="F146" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A147" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B147" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D147" s="1">
+        <v>430103051</v>
+      </c>
+      <c r="E147" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A148" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B148" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D148" s="1">
+        <v>432203039</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A149" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B149" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D149" s="1">
+        <v>432203040</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="F149" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A150" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B150" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D150" s="1">
+        <v>432202017</v>
+      </c>
+      <c r="E150" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="F150" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A151" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D151" s="1">
+        <v>430103053</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="F151" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A152" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D152" s="1">
+        <v>430103054</v>
+      </c>
+      <c r="E152" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A153" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D153" s="1">
+        <v>220103806</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="F153" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A154" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D154" s="1">
+        <v>430103055</v>
+      </c>
+      <c r="E154" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="F154" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A155" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D155" s="1">
+        <v>430103025</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="F155" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A156" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D156" s="1">
+        <v>430101062</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F156" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A157" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D157" s="1">
+        <v>430103056</v>
+      </c>
+      <c r="E157" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A158" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D158" s="1">
+        <v>430103057</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="F158" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A159" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D159" s="1">
+        <v>430103058</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F159" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A160" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D160" s="1">
+        <v>430103059</v>
+      </c>
+      <c r="E160" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="F160" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A161" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D161" s="1">
+        <v>430102071</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F161" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A162" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D162" s="1">
+        <v>432203053</v>
+      </c>
+      <c r="E162" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="F162" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A163" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D163" s="1">
+        <v>430103062</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F163" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A164" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D164" s="1">
+        <v>430103063</v>
+      </c>
+      <c r="E164" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="F164" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A165" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D165" s="1">
+        <v>432203057</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="F165" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A166" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D166" s="1">
+        <v>430103064</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="F166" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A167" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D167" s="1">
+        <v>430103065</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A168" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D168" s="1">
+        <v>430103066</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="F168" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A169" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D169" s="1">
+        <v>430103067</v>
+      </c>
+      <c r="E169" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="F169" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D170" s="1">
+        <v>432202009</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F170" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A171" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B171" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D171" s="1">
+        <v>430103068</v>
+      </c>
+      <c r="E171" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="F171" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A172" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B172" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="C172" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D172" s="1">
+        <v>432202073</v>
+      </c>
+      <c r="E172" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="F172" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A173" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D173" s="1">
+        <v>430103070</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="F173" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A174" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C174" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D174" s="1">
+        <v>432104024</v>
+      </c>
+      <c r="E174" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="F174" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A175" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D175" s="1">
+        <v>432104026</v>
+      </c>
+      <c r="E175" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="F175" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A176" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B176" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D176" s="1">
+        <v>432104027</v>
+      </c>
+      <c r="E176" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="F176" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A177" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C177" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D177" s="1">
+        <v>432104028</v>
+      </c>
+      <c r="E177" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F177" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A178" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="C178" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D178" s="1">
+        <v>432104029</v>
+      </c>
+      <c r="E178" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="F178" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A179" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C179" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D179" s="1">
+        <v>432104030</v>
+      </c>
+      <c r="E179" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F179" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A180" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C180" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D180" s="1">
+        <v>432104031</v>
+      </c>
+      <c r="E180" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A181" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B181" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="C181" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D181" s="1">
+        <v>430802057</v>
+      </c>
+      <c r="E181" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="F181" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A182" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B182" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="C182" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D182" s="1">
+        <v>432104052</v>
+      </c>
+      <c r="E182" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="F182" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A183" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B183" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C183" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D183" s="1">
+        <v>432104032</v>
+      </c>
+      <c r="E183" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="F183" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B184" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C184" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D184" s="1">
+        <v>432104006</v>
+      </c>
+      <c r="E184" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F184" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A185" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B185" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="C185" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D185" s="1">
+        <v>432104033</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="F185" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A186" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="C186" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D186" s="1">
+        <v>432104034</v>
+      </c>
+      <c r="E186" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="F186" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A187" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="C187" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D187" s="1">
+        <v>432104035</v>
+      </c>
+      <c r="E187" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F187" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A188" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C188" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D188" s="1">
+        <v>432104036</v>
+      </c>
+      <c r="E188" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="F188" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A189" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B189" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="C189" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D189" s="1">
+        <v>432104037</v>
+      </c>
+      <c r="E189" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="F189" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A190" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C190" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D190" s="1">
+        <v>432104038</v>
+      </c>
+      <c r="E190" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="F190" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A191" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D191" s="1">
+        <v>432104039</v>
+      </c>
+      <c r="E191" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="F191" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A192" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="C192" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D192" s="1">
+        <v>432104040</v>
+      </c>
+      <c r="E192" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F192" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A193" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D193" s="1">
+        <v>432104041</v>
+      </c>
+      <c r="E193" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F193" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A194" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C194" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D194" s="1">
+        <v>432104042</v>
+      </c>
+      <c r="E194" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F194" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A195" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C195" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D195" s="1">
+        <v>432104043</v>
+      </c>
+      <c r="E195" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="F195" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A196" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C196" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D196" s="1">
+        <v>432104044</v>
+      </c>
+      <c r="E196" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="F196" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A197" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="C197" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D197" s="1">
+        <v>432104045</v>
+      </c>
+      <c r="E197" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="F197" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A198" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B198" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C198" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D198" s="1">
+        <v>432104046</v>
+      </c>
+      <c r="E198" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="F198" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A199" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="C199" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D199" s="1">
+        <v>432104047</v>
+      </c>
+      <c r="E199" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="F199" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A200" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D200" s="1">
+        <v>432104048</v>
+      </c>
+      <c r="E200" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F200" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A201" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="C201" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D201" s="1">
+        <v>432104053</v>
+      </c>
+      <c r="E201" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="F201" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A202" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B202" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C202" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D202" s="1">
+        <v>432104049</v>
+      </c>
+      <c r="E202" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F202" s="3" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A203" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C203" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D203" s="1">
+        <v>432104050</v>
+      </c>
+      <c r="E203" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="F203" s="3" t="s">
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>